<commit_message>
push de la pipeline finalisée, il reste l'étape d'implementation llm
</commit_message>
<xml_diff>
--- a/BDD_raw/Maroc.xlsx
+++ b/BDD_raw/Maroc.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enquetes_Maroc" sheetId="1" r:id="R08c3e80db5ef4f40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentation" sheetId="2" r:id="R84cea7a51e1f45b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enquetes_Maroc" sheetId="1" r:id="R3c3c23f54d2641da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentation" sheetId="2" r:id="R3589eb7508a24d7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,8 +14,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
+    <x:numFmt numFmtId="201" formatCode="0.00"/>
+    <x:numFmt numFmtId="202" formatCode="0.00 &quot;€&quot;"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -54,7 +56,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -91,6 +93,18 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -113,13 +127,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EnquetesMarocTable" displayName="EnquetesMarocTable" ref="A1:E201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EnquetesMarocTable" displayName="EnquetesMarocTable" ref="A1:J201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="id_enquete"/>
     <x:tableColumn id="2" name="date_enquete"/>
     <x:tableColumn id="3" name="pays"/>
     <x:tableColumn id="4" name="code_produit"/>
-    <x:tableColumn id="5" name="commentaire_global"/>
+    <x:tableColumn id="5" name="taille_colis"/>
+    <x:tableColumn id="6" name="fragile"/>
+    <x:tableColumn id="7" name="poids_kg"/>
+    <x:tableColumn id="8" name="prix_livraison_eur"/>
+    <x:tableColumn id="9" name="statut_colis"/>
+    <x:tableColumn id="10" name="commentaire_global"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -324,7 +343,12 @@
     <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="70" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="68" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -341,6 +365,21 @@
         <x:v>code_produit</x:v>
       </x:c>
       <x:c r="E1" s="10" t="str">
+        <x:v>taille_colis</x:v>
+      </x:c>
+      <x:c r="F1" s="10" t="str">
+        <x:v>fragile</x:v>
+      </x:c>
+      <x:c r="G1" s="10" t="str">
+        <x:v>poids_kg</x:v>
+      </x:c>
+      <x:c r="H1" s="10" t="str">
+        <x:v>prix_livraison_eur</x:v>
+      </x:c>
+      <x:c r="I1" s="10" t="str">
+        <x:v>statut_colis</x:v>
+      </x:c>
+      <x:c r="J1" s="10" t="str">
         <x:v>commentaire_global</x:v>
       </x:c>
     </x:row>
@@ -358,6 +397,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E2" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F2" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G2" s="16" t="n">
+        <x:v>4.53</x:v>
+      </x:c>
+      <x:c r="H2" s="18" t="n">
+        <x:v>16.71</x:v>
+      </x:c>
+      <x:c r="I2" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J2" s="11" t="str">
         <x:v>Le colis est arrivé rapidement, mais l'emballage était légèrement abîmé.</x:v>
       </x:c>
     </x:row>
@@ -375,6 +429,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E3" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F3" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G3" s="16" t="n">
+        <x:v>1.26</x:v>
+      </x:c>
+      <x:c r="H3" s="18" t="n">
+        <x:v>9.68</x:v>
+      </x:c>
+      <x:c r="I3" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J3" s="11" t="str">
         <x:v>Le service était bon et le colis est arrivé sans dommage.</x:v>
       </x:c>
     </x:row>
@@ -392,6 +461,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="H4" s="18" t="n">
+        <x:v>5.67</x:v>
+      </x:c>
+      <x:c r="I4" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J4" s="11" t="str">
         <x:v>Tout était parfait, de la livraison à l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -409,6 +493,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G5" s="16" t="n">
+        <x:v>14.1</x:v>
+      </x:c>
+      <x:c r="H5" s="18" t="n">
+        <x:v>13.94</x:v>
+      </x:c>
+      <x:c r="I5" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J5" s="11" t="str">
         <x:v>Livraison très en retard, colis endommagé et service client impossible à joindre.</x:v>
       </x:c>
     </x:row>
@@ -426,6 +525,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E6" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G6" s="16" t="n">
+        <x:v>2.42</x:v>
+      </x:c>
+      <x:c r="H6" s="18" t="n">
+        <x:v>9.2</x:v>
+      </x:c>
+      <x:c r="I6" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J6" s="11" t="str">
         <x:v>Excellente expérience, tout s'est très bien passé.</x:v>
       </x:c>
     </x:row>
@@ -443,6 +557,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E7" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G7" s="16" t="n">
+        <x:v>0.84</x:v>
+      </x:c>
+      <x:c r="H7" s="18" t="n">
+        <x:v>5.72</x:v>
+      </x:c>
+      <x:c r="I7" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J7" s="11" t="str">
         <x:v>Très bonne expérience, avec une livraison ponctuelle et un colis impeccable.</x:v>
       </x:c>
     </x:row>
@@ -460,6 +589,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E8" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G8" s="16" t="n">
+        <x:v>0.91</x:v>
+      </x:c>
+      <x:c r="H8" s="18" t="n">
+        <x:v>5.76</x:v>
+      </x:c>
+      <x:c r="I8" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J8" s="11" t="str">
         <x:v>Le colis a bien été reçu, avec un léger retard sans conséquence importante.</x:v>
       </x:c>
     </x:row>
@@ -477,6 +621,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E9" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G9" s="16" t="n">
+        <x:v>4.86</x:v>
+      </x:c>
+      <x:c r="H9" s="18" t="n">
+        <x:v>11.91</x:v>
+      </x:c>
+      <x:c r="I9" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J9" s="11" t="str">
         <x:v>Je suis pleinement satisfait, le service a été rapide et professionnel.</x:v>
       </x:c>
     </x:row>
@@ -494,6 +653,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E10" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G10" s="16" t="n">
+        <x:v>4.14</x:v>
+      </x:c>
+      <x:c r="H10" s="18" t="n">
+        <x:v>7.77</x:v>
+      </x:c>
+      <x:c r="I10" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J10" s="11" t="str">
         <x:v>Je suis plutôt insatisfait, surtout à cause du délai de livraison.</x:v>
       </x:c>
     </x:row>
@@ -511,6 +685,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E11" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G11" s="16" t="n">
+        <x:v>1.23</x:v>
+      </x:c>
+      <x:c r="H11" s="18" t="n">
+        <x:v>5.96</x:v>
+      </x:c>
+      <x:c r="I11" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J11" s="11" t="str">
         <x:v>Expérience décevante dans l'ensemble, malgré un colis reçu en bon état.</x:v>
       </x:c>
     </x:row>
@@ -528,6 +717,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E12" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F12" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G12" s="16" t="n">
+        <x:v>3.75</x:v>
+      </x:c>
+      <x:c r="H12" s="18" t="n">
+        <x:v>7.53</x:v>
+      </x:c>
+      <x:c r="I12" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J12" s="11" t="str">
         <x:v>Très bonne expérience, avec une livraison ponctuelle et un colis impeccable.</x:v>
       </x:c>
     </x:row>
@@ -545,6 +749,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E13" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F13" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G13" s="16" t="n">
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="H13" s="18" t="n">
+        <x:v>5.34</x:v>
+      </x:c>
+      <x:c r="I13" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J13" s="11" t="str">
         <x:v>Livraison très rapide, colis en parfait état et livreur très professionnel.</x:v>
       </x:c>
     </x:row>
@@ -562,6 +781,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E14" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F14" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G14" s="16" t="n">
+        <x:v>0.44</x:v>
+      </x:c>
+      <x:c r="H14" s="18" t="n">
+        <x:v>5.47</x:v>
+      </x:c>
+      <x:c r="I14" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J14" s="11" t="str">
         <x:v>Excellente expérience, tout s'est très bien passé.</x:v>
       </x:c>
     </x:row>
@@ -579,6 +813,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E15" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F15" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G15" s="16" t="n">
+        <x:v>8.09</x:v>
+      </x:c>
+      <x:c r="H15" s="18" t="n">
+        <x:v>12.72</x:v>
+      </x:c>
+      <x:c r="I15" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J15" s="11" t="str">
         <x:v>Le colis est arrivé intact mais le suivi et le service client n'étaient pas satisfaisants.</x:v>
       </x:c>
     </x:row>
@@ -596,6 +845,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E16" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F16" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G16" s="16" t="n">
+        <x:v>1.45</x:v>
+      </x:c>
+      <x:c r="H16" s="18" t="n">
+        <x:v>6.1</x:v>
+      </x:c>
+      <x:c r="I16" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J16" s="11" t="str">
         <x:v>Expérience correcte dans l'ensemble, mais le service client pourrait être plus réactif.</x:v>
       </x:c>
     </x:row>
@@ -612,7 +876,22 @@
       <x:c r="D17" s="11" t="str">
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
-      <x:c r="E17" s="11"/>
+      <x:c r="E17" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F17" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G17" s="16" t="n">
+        <x:v>0.87</x:v>
+      </x:c>
+      <x:c r="H17" s="18" t="n">
+        <x:v>5.74</x:v>
+      </x:c>
+      <x:c r="I17" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J17" s="11"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="11" t="str">
@@ -628,6 +907,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E18" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F18" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G18" s="16" t="n">
+        <x:v>2.27</x:v>
+      </x:c>
+      <x:c r="H18" s="18" t="n">
+        <x:v>6.61</x:v>
+      </x:c>
+      <x:c r="I18" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J18" s="11" t="str">
         <x:v>Expérience positive dans l'ensemble, avec un colis reçu proprement et dans les temps.</x:v>
       </x:c>
     </x:row>
@@ -644,7 +938,22 @@
       <x:c r="D19" s="11" t="str">
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
-      <x:c r="E19" s="11"/>
+      <x:c r="E19" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F19" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G19" s="16" t="n">
+        <x:v>11.19</x:v>
+      </x:c>
+      <x:c r="H19" s="18" t="n">
+        <x:v>15.84</x:v>
+      </x:c>
+      <x:c r="I19" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J19" s="11"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="11" t="str">
@@ -660,6 +969,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E20" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F20" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G20" s="16" t="n">
+        <x:v>5.56</x:v>
+      </x:c>
+      <x:c r="H20" s="18" t="n">
+        <x:v>8.65</x:v>
+      </x:c>
+      <x:c r="I20" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J20" s="11" t="str">
         <x:v>La livraison s'est passée normalement et le colis était en bon état.</x:v>
       </x:c>
     </x:row>
@@ -677,6 +1001,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F21" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G21" s="16" t="n">
+        <x:v>2.06</x:v>
+      </x:c>
+      <x:c r="H21" s="18" t="n">
+        <x:v>6.48</x:v>
+      </x:c>
+      <x:c r="I21" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J21" s="11" t="str">
         <x:v>Bonne prise en charge, livraison correcte et livreur professionnel.</x:v>
       </x:c>
     </x:row>
@@ -694,6 +1033,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E22" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F22" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G22" s="16" t="n">
+        <x:v>5.72</x:v>
+      </x:c>
+      <x:c r="H22" s="18" t="n">
+        <x:v>14.95</x:v>
+      </x:c>
+      <x:c r="I22" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J22" s="11" t="str">
         <x:v>Le colis a bien été reçu, avec un léger retard sans conséquence importante.</x:v>
       </x:c>
     </x:row>
@@ -711,6 +1065,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E23" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F23" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G23" s="16" t="n">
+        <x:v>9.18</x:v>
+      </x:c>
+      <x:c r="H23" s="18" t="n">
+        <x:v>19.59</x:v>
+      </x:c>
+      <x:c r="I23" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J23" s="11" t="str">
         <x:v>La livraison a été lente et les réponses du service client peu utiles.</x:v>
       </x:c>
     </x:row>
@@ -728,6 +1097,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E24" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F24" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G24" s="16" t="n">
+        <x:v>0.37</x:v>
+      </x:c>
+      <x:c r="H24" s="18" t="n">
+        <x:v>5.43</x:v>
+      </x:c>
+      <x:c r="I24" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J24" s="11" t="str">
         <x:v>Très satisfait : livraison rapide, livreur courtois et service client efficace.</x:v>
       </x:c>
     </x:row>
@@ -745,6 +1129,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E25" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F25" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G25" s="16" t="n">
+        <x:v>7.14</x:v>
+      </x:c>
+      <x:c r="H25" s="18" t="n">
+        <x:v>9.63</x:v>
+      </x:c>
+      <x:c r="I25" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J25" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -762,6 +1161,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E26" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F26" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G26" s="16" t="n">
+        <x:v>1.28</x:v>
+      </x:c>
+      <x:c r="H26" s="18" t="n">
+        <x:v>5.99</x:v>
+      </x:c>
+      <x:c r="I26" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J26" s="11" t="str">
         <x:v>Bonne expérience dans l'ensemble, malgré un léger retard.</x:v>
       </x:c>
     </x:row>
@@ -779,6 +1193,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E27" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F27" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G27" s="16" t="n">
+        <x:v>3.13</x:v>
+      </x:c>
+      <x:c r="H27" s="18" t="n">
+        <x:v>9.64</x:v>
+      </x:c>
+      <x:c r="I27" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J27" s="11" t="str">
         <x:v>Le service était bon et le colis est arrivé sans dommage.</x:v>
       </x:c>
     </x:row>
@@ -796,6 +1225,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E28" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F28" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G28" s="16" t="n">
+        <x:v>2.7</x:v>
+      </x:c>
+      <x:c r="H28" s="18" t="n">
+        <x:v>13.07</x:v>
+      </x:c>
+      <x:c r="I28" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J28" s="11" t="str">
         <x:v>Livraison très en retard, colis endommagé et service client impossible à joindre.</x:v>
       </x:c>
     </x:row>
@@ -813,6 +1257,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E29" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F29" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G29" s="16" t="n">
+        <x:v>1.44</x:v>
+      </x:c>
+      <x:c r="H29" s="18" t="n">
+        <x:v>6.09</x:v>
+      </x:c>
+      <x:c r="I29" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J29" s="11" t="str">
         <x:v>Bonne expérience dans l'ensemble, malgré un léger retard.</x:v>
       </x:c>
     </x:row>
@@ -830,6 +1289,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E30" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F30" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G30" s="16" t="n">
+        <x:v>2.56</x:v>
+      </x:c>
+      <x:c r="H30" s="18" t="n">
+        <x:v>6.79</x:v>
+      </x:c>
+      <x:c r="I30" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J30" s="11" t="str">
         <x:v>Bonne prise en charge, livraison correcte et livreur professionnel.</x:v>
       </x:c>
     </x:row>
@@ -847,6 +1321,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E31" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F31" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G31" s="16" t="n">
+        <x:v>0.43</x:v>
+      </x:c>
+      <x:c r="H31" s="18" t="n">
+        <x:v>5.47</x:v>
+      </x:c>
+      <x:c r="I31" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J31" s="11" t="str">
         <x:v>Expérience décevante dans l'ensemble, malgré un colis reçu en bon état.</x:v>
       </x:c>
     </x:row>
@@ -864,6 +1353,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E32" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F32" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G32" s="16" t="n">
+        <x:v>1.06</x:v>
+      </x:c>
+      <x:c r="H32" s="18" t="n">
+        <x:v>5.86</x:v>
+      </x:c>
+      <x:c r="I32" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J32" s="11" t="str">
         <x:v>Service excellent, colis livré rapidement et sans aucun problème.</x:v>
       </x:c>
     </x:row>
@@ -881,6 +1385,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E33" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F33" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G33" s="16" t="n">
+        <x:v>1.76</x:v>
+      </x:c>
+      <x:c r="H33" s="18" t="n">
+        <x:v>12.49</x:v>
+      </x:c>
+      <x:c r="I33" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J33" s="11" t="str">
         <x:v>Bonne expérience dans l'ensemble, malgré un léger retard.</x:v>
       </x:c>
     </x:row>
@@ -898,6 +1417,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E34" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F34" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G34" s="16" t="n">
+        <x:v>16.31</x:v>
+      </x:c>
+      <x:c r="H34" s="18" t="n">
+        <x:v>17.81</x:v>
+      </x:c>
+      <x:c r="I34" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J34" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -915,6 +1449,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E35" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F35" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G35" s="16" t="n">
+        <x:v>2.06</x:v>
+      </x:c>
+      <x:c r="H35" s="18" t="n">
+        <x:v>8.98</x:v>
+      </x:c>
+      <x:c r="I35" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J35" s="11" t="str">
         <x:v>Expérience correcte dans l'ensemble, mais le service client pourrait être plus réactif.</x:v>
       </x:c>
     </x:row>
@@ -932,6 +1481,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E36" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F36" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G36" s="16" t="n">
+        <x:v>2.28</x:v>
+      </x:c>
+      <x:c r="H36" s="18" t="n">
+        <x:v>9.11</x:v>
+      </x:c>
+      <x:c r="I36" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J36" s="11" t="str">
         <x:v>Service globalement moyen, ni particulièrement bon ni mauvais.</x:v>
       </x:c>
     </x:row>
@@ -949,6 +1513,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E37" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F37" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G37" s="16" t="n">
+        <x:v>5.41</x:v>
+      </x:c>
+      <x:c r="H37" s="18" t="n">
+        <x:v>19.75</x:v>
+      </x:c>
+      <x:c r="I37" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J37" s="11" t="str">
         <x:v>Rien de particulier à signaler, le service était acceptable.</x:v>
       </x:c>
     </x:row>
@@ -966,6 +1545,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E38" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F38" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G38" s="16" t="n">
+        <x:v>1.76</x:v>
+      </x:c>
+      <x:c r="H38" s="18" t="n">
+        <x:v>6.29</x:v>
+      </x:c>
+      <x:c r="I38" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J38" s="11" t="str">
         <x:v>Le service était bon et le colis est arrivé sans dommage.</x:v>
       </x:c>
     </x:row>
@@ -983,6 +1577,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E39" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F39" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G39" s="16" t="n">
+        <x:v>2.81</x:v>
+      </x:c>
+      <x:c r="H39" s="18" t="n">
+        <x:v>13.14</x:v>
+      </x:c>
+      <x:c r="I39" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J39" s="11" t="str">
         <x:v>Très bonne expérience, avec une livraison ponctuelle et un colis impeccable.</x:v>
       </x:c>
     </x:row>
@@ -1000,6 +1609,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E40" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F40" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G40" s="16" t="n">
+        <x:v>1.14</x:v>
+      </x:c>
+      <x:c r="H40" s="18" t="n">
+        <x:v>5.91</x:v>
+      </x:c>
+      <x:c r="I40" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J40" s="11" t="str">
         <x:v>Je suis pleinement satisfait, le service a été rapide et professionnel.</x:v>
       </x:c>
     </x:row>
@@ -1017,6 +1641,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E41" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F41" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G41" s="16" t="n">
+        <x:v>5.91</x:v>
+      </x:c>
+      <x:c r="H41" s="18" t="n">
+        <x:v>8.86</x:v>
+      </x:c>
+      <x:c r="I41" s="11" t="str">
+        <x:v>Retourné</x:v>
+      </x:c>
+      <x:c r="J41" s="11" t="str">
         <x:v>Le service a été mauvais du début à la fin, avec beaucoup de retard et un colis abîmé.</x:v>
       </x:c>
     </x:row>
@@ -1034,6 +1673,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E42" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F42" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G42" s="16" t="n">
+        <x:v>12.96</x:v>
+      </x:c>
+      <x:c r="H42" s="18" t="n">
+        <x:v>16.94</x:v>
+      </x:c>
+      <x:c r="I42" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J42" s="11" t="str">
         <x:v>Le colis est arrivé correctement, même si l'expérience n'avait rien d'exceptionnel.</x:v>
       </x:c>
     </x:row>
@@ -1050,7 +1704,22 @@
       <x:c r="D43" s="11" t="str">
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
-      <x:c r="E43" s="11"/>
+      <x:c r="E43" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F43" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G43" s="16" t="n">
+        <x:v>3.64</x:v>
+      </x:c>
+      <x:c r="H43" s="18" t="n">
+        <x:v>11.16</x:v>
+      </x:c>
+      <x:c r="I43" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J43" s="11"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="11" t="str">
@@ -1066,6 +1735,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E44" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F44" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G44" s="16" t="n">
+        <x:v>1.45</x:v>
+      </x:c>
+      <x:c r="H44" s="18" t="n">
+        <x:v>9.8</x:v>
+      </x:c>
+      <x:c r="I44" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J44" s="11" t="str">
         <x:v>La livraison était correcte, sans problème particulier.</x:v>
       </x:c>
     </x:row>
@@ -1083,6 +1767,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E45" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F45" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G45" s="16" t="n">
+        <x:v>5.84</x:v>
+      </x:c>
+      <x:c r="H45" s="18" t="n">
+        <x:v>8.82</x:v>
+      </x:c>
+      <x:c r="I45" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J45" s="11" t="str">
         <x:v>Le colis est arrivé à temps et le livreur était professionnel.</x:v>
       </x:c>
     </x:row>
@@ -1100,6 +1799,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E46" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F46" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G46" s="16" t="n">
+        <x:v>2.86</x:v>
+      </x:c>
+      <x:c r="H46" s="18" t="n">
+        <x:v>13.17</x:v>
+      </x:c>
+      <x:c r="I46" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J46" s="11" t="str">
         <x:v>Le colis est arrivé intact mais le suivi et le service client n'étaient pas satisfaisants.</x:v>
       </x:c>
     </x:row>
@@ -1116,7 +1830,22 @@
       <x:c r="D47" s="11" t="str">
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
-      <x:c r="E47" s="11"/>
+      <x:c r="E47" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F47" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G47" s="16" t="n">
+        <x:v>0.54</x:v>
+      </x:c>
+      <x:c r="H47" s="18" t="n">
+        <x:v>5.53</x:v>
+      </x:c>
+      <x:c r="I47" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J47" s="11"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="11" t="str">
@@ -1132,6 +1861,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E48" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F48" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G48" s="16" t="n">
+        <x:v>11.22</x:v>
+      </x:c>
+      <x:c r="H48" s="18" t="n">
+        <x:v>18.36</x:v>
+      </x:c>
+      <x:c r="I48" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J48" s="11" t="str">
         <x:v>Le service était bon et le colis est arrivé sans dommage.</x:v>
       </x:c>
     </x:row>
@@ -1149,6 +1893,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E49" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F49" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G49" s="16" t="n">
+        <x:v>14.49</x:v>
+      </x:c>
+      <x:c r="H49" s="18" t="n">
+        <x:v>25.38</x:v>
+      </x:c>
+      <x:c r="I49" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J49" s="11" t="str">
         <x:v>Service client efficace, même si la livraison a pris plus de temps que prévu.</x:v>
       </x:c>
     </x:row>
@@ -1166,6 +1925,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E50" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F50" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G50" s="16" t="n">
+        <x:v>3.16</x:v>
+      </x:c>
+      <x:c r="H50" s="18" t="n">
+        <x:v>10.86</x:v>
+      </x:c>
+      <x:c r="I50" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J50" s="11" t="str">
         <x:v>Expérience très insatisfaisante, livraison tardive et mauvaise prise en charge du service client.</x:v>
       </x:c>
     </x:row>
@@ -1183,6 +1957,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E51" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F51" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G51" s="16" t="n">
+        <x:v>5.59</x:v>
+      </x:c>
+      <x:c r="H51" s="18" t="n">
+        <x:v>8.67</x:v>
+      </x:c>
+      <x:c r="I51" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J51" s="11" t="str">
         <x:v>La livraison s'est passée normalement et le colis était en bon état.</x:v>
       </x:c>
     </x:row>
@@ -1200,6 +1989,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E52" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F52" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G52" s="16" t="n">
+        <x:v>0.62</x:v>
+      </x:c>
+      <x:c r="H52" s="18" t="n">
+        <x:v>9.28</x:v>
+      </x:c>
+      <x:c r="I52" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J52" s="11" t="str">
         <x:v>Expérience correcte dans l'ensemble, mais le service client pourrait être plus réactif.</x:v>
       </x:c>
     </x:row>
@@ -1217,6 +2021,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E53" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F53" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G53" s="16" t="n">
+        <x:v>3.78</x:v>
+      </x:c>
+      <x:c r="H53" s="18" t="n">
+        <x:v>13.74</x:v>
+      </x:c>
+      <x:c r="I53" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J53" s="11" t="str">
         <x:v>Le colis était correct mais la livraison a pris trop de temps.</x:v>
       </x:c>
     </x:row>
@@ -1234,6 +2053,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E54" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F54" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G54" s="16" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="H54" s="18" t="n">
+        <x:v>5.7</x:v>
+      </x:c>
+      <x:c r="I54" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J54" s="11" t="str">
         <x:v>Très bonne expérience, avec une livraison ponctuelle et un colis impeccable.</x:v>
       </x:c>
     </x:row>
@@ -1250,7 +2084,22 @@
       <x:c r="D55" s="11" t="str">
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
-      <x:c r="E55" s="11"/>
+      <x:c r="E55" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F55" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G55" s="16" t="n">
+        <x:v>16.04</x:v>
+      </x:c>
+      <x:c r="H55" s="18" t="n">
+        <x:v>26.34</x:v>
+      </x:c>
+      <x:c r="I55" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J55" s="11"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="11" t="str">
@@ -1266,6 +2115,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E56" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F56" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G56" s="16" t="n">
+        <x:v>1.29</x:v>
+      </x:c>
+      <x:c r="H56" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I56" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J56" s="11" t="str">
         <x:v>Bonne prise en charge, livraison correcte et livreur professionnel.</x:v>
       </x:c>
     </x:row>
@@ -1283,6 +2147,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E57" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F57" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G57" s="16" t="n">
+        <x:v>1.86</x:v>
+      </x:c>
+      <x:c r="H57" s="18" t="n">
+        <x:v>10.05</x:v>
+      </x:c>
+      <x:c r="I57" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J57" s="11" t="str">
         <x:v>Je suis plutôt insatisfait, surtout à cause du délai de livraison.</x:v>
       </x:c>
     </x:row>
@@ -1300,6 +2179,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E58" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F58" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G58" s="16" t="n">
+        <x:v>1.7</x:v>
+      </x:c>
+      <x:c r="H58" s="18" t="n">
+        <x:v>6.25</x:v>
+      </x:c>
+      <x:c r="I58" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J58" s="11" t="str">
         <x:v>Livraison très rapide, colis en parfait état et livreur très professionnel.</x:v>
       </x:c>
     </x:row>
@@ -1317,6 +2211,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E59" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F59" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G59" s="16" t="n">
+        <x:v>3.07</x:v>
+      </x:c>
+      <x:c r="H59" s="18" t="n">
+        <x:v>18.3</x:v>
+      </x:c>
+      <x:c r="I59" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J59" s="11" t="str">
         <x:v>Le colis a été livré dans de bonnes conditions et le service client a répondu rapidement.</x:v>
       </x:c>
     </x:row>
@@ -1334,6 +2243,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E60" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F60" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G60" s="16" t="n">
+        <x:v>1.11</x:v>
+      </x:c>
+      <x:c r="H60" s="18" t="n">
+        <x:v>12.09</x:v>
+      </x:c>
+      <x:c r="I60" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J60" s="11" t="str">
         <x:v>La livraison s'est mal passée, même si le colis était en bon état.</x:v>
       </x:c>
     </x:row>
@@ -1351,6 +2275,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E61" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F61" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G61" s="16" t="n">
+        <x:v>8.65</x:v>
+      </x:c>
+      <x:c r="H61" s="18" t="n">
+        <x:v>10.56</x:v>
+      </x:c>
+      <x:c r="I61" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J61" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -1368,6 +2307,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E62" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F62" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G62" s="16" t="n">
+        <x:v>7.78</x:v>
+      </x:c>
+      <x:c r="H62" s="18" t="n">
+        <x:v>18.72</x:v>
+      </x:c>
+      <x:c r="I62" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J62" s="11" t="str">
         <x:v>Le livreur était courtois et le colis intact, mais le suivi de livraison manquait de précision.</x:v>
       </x:c>
     </x:row>
@@ -1385,6 +2339,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E63" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F63" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G63" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H63" s="18" t="n">
+        <x:v>5.82</x:v>
+      </x:c>
+      <x:c r="I63" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J63" s="11" t="str">
         <x:v>Livraison rapide mais colis légèrement endommagé.</x:v>
       </x:c>
     </x:row>
@@ -1402,6 +2371,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E64" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F64" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G64" s="16" t="n">
+        <x:v>8.3</x:v>
+      </x:c>
+      <x:c r="H64" s="18" t="n">
+        <x:v>10.35</x:v>
+      </x:c>
+      <x:c r="I64" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J64" s="11" t="str">
         <x:v>Je suis très déçu : le colis a été livré tard et en mauvais état.</x:v>
       </x:c>
     </x:row>
@@ -1419,6 +2403,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E65" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F65" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G65" s="16" t="n">
+        <x:v>17.76</x:v>
+      </x:c>
+      <x:c r="H65" s="18" t="n">
+        <x:v>24.91</x:v>
+      </x:c>
+      <x:c r="I65" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J65" s="11" t="str">
         <x:v>Le colis est arrivé à temps et le livreur était professionnel.</x:v>
       </x:c>
     </x:row>
@@ -1436,6 +2435,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E66" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F66" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G66" s="16" t="n">
+        <x:v>13.19</x:v>
+      </x:c>
+      <x:c r="H66" s="18" t="n">
+        <x:v>19.58</x:v>
+      </x:c>
+      <x:c r="I66" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J66" s="11" t="str">
         <x:v>Service globalement moyen, ni particulièrement bon ni mauvais.</x:v>
       </x:c>
     </x:row>
@@ -1453,6 +2467,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E67" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F67" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G67" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H67" s="18" t="n">
+        <x:v>5.82</x:v>
+      </x:c>
+      <x:c r="I67" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J67" s="11" t="str">
         <x:v>Le colis a été livré dans de bonnes conditions et le service client a répondu rapidement.</x:v>
       </x:c>
     </x:row>
@@ -1470,6 +2499,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E68" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F68" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G68" s="16" t="n">
+        <x:v>4.39</x:v>
+      </x:c>
+      <x:c r="H68" s="18" t="n">
+        <x:v>7.92</x:v>
+      </x:c>
+      <x:c r="I68" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J68" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -1487,6 +2531,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E69" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F69" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G69" s="16" t="n">
+        <x:v>2.34</x:v>
+      </x:c>
+      <x:c r="H69" s="18" t="n">
+        <x:v>6.65</x:v>
+      </x:c>
+      <x:c r="I69" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J69" s="11" t="str">
         <x:v>Expérience décevante dans l'ensemble, malgré un colis reçu en bon état.</x:v>
       </x:c>
     </x:row>
@@ -1504,6 +2563,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E70" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F70" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G70" s="16" t="n">
+        <x:v>3.71</x:v>
+      </x:c>
+      <x:c r="H70" s="18" t="n">
+        <x:v>11.2</x:v>
+      </x:c>
+      <x:c r="I70" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J70" s="11" t="str">
         <x:v>La livraison a été lente et les réponses du service client peu utiles.</x:v>
       </x:c>
     </x:row>
@@ -1521,6 +2595,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E71" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F71" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G71" s="16" t="n">
+        <x:v>1.16</x:v>
+      </x:c>
+      <x:c r="H71" s="18" t="n">
+        <x:v>8.42</x:v>
+      </x:c>
+      <x:c r="I71" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J71" s="11" t="str">
         <x:v>Bonne expérience dans l'ensemble, malgré un léger retard.</x:v>
       </x:c>
     </x:row>
@@ -1538,6 +2627,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E72" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F72" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G72" s="16" t="n">
+        <x:v>1.12</x:v>
+      </x:c>
+      <x:c r="H72" s="18" t="n">
+        <x:v>14.59</x:v>
+      </x:c>
+      <x:c r="I72" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J72" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -1555,6 +2659,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E73" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F73" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G73" s="16" t="n">
+        <x:v>10.95</x:v>
+      </x:c>
+      <x:c r="H73" s="18" t="n">
+        <x:v>11.99</x:v>
+      </x:c>
+      <x:c r="I73" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J73" s="11" t="str">
         <x:v>Très satisfait : livraison rapide, livreur courtois et service client efficace.</x:v>
       </x:c>
     </x:row>
@@ -1572,6 +2691,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E74" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F74" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G74" s="16" t="n">
+        <x:v>4.19</x:v>
+      </x:c>
+      <x:c r="H74" s="18" t="n">
+        <x:v>16.5</x:v>
+      </x:c>
+      <x:c r="I74" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J74" s="11" t="str">
         <x:v>La livraison était correcte, sans problème particulier.</x:v>
       </x:c>
     </x:row>
@@ -1589,6 +2723,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E75" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F75" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G75" s="16" t="n">
+        <x:v>15.34</x:v>
+      </x:c>
+      <x:c r="H75" s="18" t="n">
+        <x:v>18.41</x:v>
+      </x:c>
+      <x:c r="I75" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J75" s="11" t="str">
         <x:v>Le colis est arrivé plusieurs jours en retard et le support n'a pas résolu mon problème.</x:v>
       </x:c>
     </x:row>
@@ -1606,6 +2755,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E76" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F76" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G76" s="16" t="n">
+        <x:v>5.4</x:v>
+      </x:c>
+      <x:c r="H76" s="18" t="n">
+        <x:v>8.55</x:v>
+      </x:c>
+      <x:c r="I76" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J76" s="11" t="str">
         <x:v>Très mauvaise expérience, livraison tardive et colis abîmé à l'arrivée.</x:v>
       </x:c>
     </x:row>
@@ -1623,6 +2787,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E77" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F77" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G77" s="16" t="n">
+        <x:v>1.97</x:v>
+      </x:c>
+      <x:c r="H77" s="18" t="n">
+        <x:v>6.42</x:v>
+      </x:c>
+      <x:c r="I77" s="11" t="str">
+        <x:v>Retourné</x:v>
+      </x:c>
+      <x:c r="J77" s="11" t="str">
         <x:v>Bonne prise en charge, livraison correcte et livreur professionnel.</x:v>
       </x:c>
     </x:row>
@@ -1640,6 +2819,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E78" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F78" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G78" s="16" t="n">
+        <x:v>6.15</x:v>
+      </x:c>
+      <x:c r="H78" s="18" t="n">
+        <x:v>9.01</x:v>
+      </x:c>
+      <x:c r="I78" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J78" s="11" t="str">
         <x:v>Bonne expérience dans l'ensemble, malgré un léger retard.</x:v>
       </x:c>
     </x:row>
@@ -1657,6 +2851,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E79" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F79" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G79" s="16" t="n">
+        <x:v>4.45</x:v>
+      </x:c>
+      <x:c r="H79" s="18" t="n">
+        <x:v>7.96</x:v>
+      </x:c>
+      <x:c r="I79" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J79" s="11" t="str">
         <x:v>Expérience correcte dans l'ensemble, mais le service client pourrait être plus réactif.</x:v>
       </x:c>
     </x:row>
@@ -1674,6 +2883,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E80" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F80" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G80" s="16" t="n">
+        <x:v>1.48</x:v>
+      </x:c>
+      <x:c r="H80" s="18" t="n">
+        <x:v>9.82</x:v>
+      </x:c>
+      <x:c r="I80" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J80" s="11" t="str">
         <x:v>Livraison très rapide, colis en parfait état et livreur très professionnel.</x:v>
       </x:c>
     </x:row>
@@ -1691,6 +2915,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E81" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F81" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G81" s="16" t="n">
+        <x:v>8.21</x:v>
+      </x:c>
+      <x:c r="H81" s="18" t="n">
+        <x:v>13.99</x:v>
+      </x:c>
+      <x:c r="I81" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J81" s="11" t="str">
         <x:v>La livraison était correcte, sans problème particulier.</x:v>
       </x:c>
     </x:row>
@@ -1708,6 +2947,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E82" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F82" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G82" s="16" t="n">
+        <x:v>4.24</x:v>
+      </x:c>
+      <x:c r="H82" s="18" t="n">
+        <x:v>11.53</x:v>
+      </x:c>
+      <x:c r="I82" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J82" s="11" t="str">
         <x:v>Service excellent, colis livré rapidement et sans aucun problème.</x:v>
       </x:c>
     </x:row>
@@ -1725,6 +2979,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E83" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F83" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G83" s="16" t="n">
+        <x:v>8.16</x:v>
+      </x:c>
+      <x:c r="H83" s="18" t="n">
+        <x:v>16.46</x:v>
+      </x:c>
+      <x:c r="I83" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J83" s="11" t="str">
         <x:v>Le colis a été livré dans de bonnes conditions et le service client a répondu rapidement.</x:v>
       </x:c>
     </x:row>
@@ -1742,6 +3011,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E84" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F84" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G84" s="16" t="n">
+        <x:v>4.89</x:v>
+      </x:c>
+      <x:c r="H84" s="18" t="n">
+        <x:v>10.73</x:v>
+      </x:c>
+      <x:c r="I84" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J84" s="11" t="str">
         <x:v>Expérience positive dans l'ensemble, avec un colis reçu proprement et dans les temps.</x:v>
       </x:c>
     </x:row>
@@ -1759,6 +3043,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E85" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F85" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G85" s="16" t="n">
+        <x:v>3.55</x:v>
+      </x:c>
+      <x:c r="H85" s="18" t="n">
+        <x:v>18.6</x:v>
+      </x:c>
+      <x:c r="I85" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J85" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -1776,6 +3075,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E86" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F86" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G86" s="16" t="n">
+        <x:v>2.04</x:v>
+      </x:c>
+      <x:c r="H86" s="18" t="n">
+        <x:v>6.46</x:v>
+      </x:c>
+      <x:c r="I86" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J86" s="11" t="str">
         <x:v>Très satisfait : livraison rapide, livreur courtois et service client efficace.</x:v>
       </x:c>
     </x:row>
@@ -1793,6 +3107,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E87" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F87" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G87" s="16" t="n">
+        <x:v>4.45</x:v>
+      </x:c>
+      <x:c r="H87" s="18" t="n">
+        <x:v>7.96</x:v>
+      </x:c>
+      <x:c r="I87" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J87" s="11" t="str">
         <x:v>La livraison était correcte, sans problème particulier.</x:v>
       </x:c>
     </x:row>
@@ -1810,6 +3139,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E88" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F88" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G88" s="16" t="n">
+        <x:v>5.67</x:v>
+      </x:c>
+      <x:c r="H88" s="18" t="n">
+        <x:v>19.92</x:v>
+      </x:c>
+      <x:c r="I88" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J88" s="11" t="str">
         <x:v>Tout était parfait, de la livraison à l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -1827,6 +3171,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E89" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F89" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G89" s="16" t="n">
+        <x:v>0.56</x:v>
+      </x:c>
+      <x:c r="H89" s="18" t="n">
+        <x:v>5.55</x:v>
+      </x:c>
+      <x:c r="I89" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J89" s="11" t="str">
         <x:v>Le colis est arrivé plus tôt que prévu, parfaitement emballé et en excellent état.</x:v>
       </x:c>
     </x:row>
@@ -1844,6 +3203,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E90" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F90" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G90" s="16" t="n">
+        <x:v>3.92</x:v>
+      </x:c>
+      <x:c r="H90" s="18" t="n">
+        <x:v>7.63</x:v>
+      </x:c>
+      <x:c r="I90" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J90" s="11" t="str">
         <x:v>Livraison très rapide, colis en parfait état et livreur très professionnel.</x:v>
       </x:c>
     </x:row>
@@ -1861,6 +3235,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E91" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F91" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G91" s="16" t="n">
+        <x:v>5.27</x:v>
+      </x:c>
+      <x:c r="H91" s="18" t="n">
+        <x:v>8.47</x:v>
+      </x:c>
+      <x:c r="I91" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J91" s="11" t="str">
         <x:v>Service excellent, colis livré rapidement et sans aucun problème.</x:v>
       </x:c>
     </x:row>
@@ -1877,7 +3266,22 @@
       <x:c r="D92" s="11" t="str">
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
-      <x:c r="E92" s="11"/>
+      <x:c r="E92" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F92" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G92" s="16" t="n">
+        <x:v>0.54</x:v>
+      </x:c>
+      <x:c r="H92" s="18" t="n">
+        <x:v>8.03</x:v>
+      </x:c>
+      <x:c r="I92" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J92" s="11"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="11" t="str">
@@ -1892,7 +3296,22 @@
       <x:c r="D93" s="11" t="str">
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
-      <x:c r="E93" s="11"/>
+      <x:c r="E93" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F93" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G93" s="16" t="n">
+        <x:v>4.94</x:v>
+      </x:c>
+      <x:c r="H93" s="18" t="n">
+        <x:v>11.96</x:v>
+      </x:c>
+      <x:c r="I93" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J93" s="11"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="11" t="str">
@@ -1908,6 +3327,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E94" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F94" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G94" s="16" t="n">
+        <x:v>5.66</x:v>
+      </x:c>
+      <x:c r="H94" s="18" t="n">
+        <x:v>8.71</x:v>
+      </x:c>
+      <x:c r="I94" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J94" s="11" t="str">
         <x:v>Expérience décevante dans l'ensemble, malgré un colis reçu en bon état.</x:v>
       </x:c>
     </x:row>
@@ -1925,6 +3359,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E95" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F95" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G95" s="16" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="H95" s="18" t="n">
+        <x:v>5.57</x:v>
+      </x:c>
+      <x:c r="I95" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J95" s="11" t="str">
         <x:v>Le colis est arrivé intact mais le suivi et le service client n'étaient pas satisfaisants.</x:v>
       </x:c>
     </x:row>
@@ -1942,6 +3391,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E96" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F96" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G96" s="16" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="H96" s="18" t="n">
+        <x:v>7.25</x:v>
+      </x:c>
+      <x:c r="I96" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J96" s="11" t="str">
         <x:v>Le colis est arrivé correctement, même si l'expérience n'avait rien d'exceptionnel.</x:v>
       </x:c>
     </x:row>
@@ -1959,6 +3423,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E97" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F97" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G97" s="16" t="n">
+        <x:v>1.62</x:v>
+      </x:c>
+      <x:c r="H97" s="18" t="n">
+        <x:v>8.7</x:v>
+      </x:c>
+      <x:c r="I97" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J97" s="11" t="str">
         <x:v>Livraison très en retard, colis endommagé et service client impossible à joindre.</x:v>
       </x:c>
     </x:row>
@@ -1976,6 +3455,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E98" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F98" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G98" s="16" t="n">
+        <x:v>4.84</x:v>
+      </x:c>
+      <x:c r="H98" s="18" t="n">
+        <x:v>16.9</x:v>
+      </x:c>
+      <x:c r="I98" s="11" t="str">
+        <x:v>Retourné</x:v>
+      </x:c>
+      <x:c r="J98" s="11" t="str">
         <x:v>La livraison s'est passée normalement et le colis était en bon état.</x:v>
       </x:c>
     </x:row>
@@ -1993,6 +3487,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E99" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F99" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G99" s="16" t="n">
+        <x:v>2.92</x:v>
+      </x:c>
+      <x:c r="H99" s="18" t="n">
+        <x:v>9.51</x:v>
+      </x:c>
+      <x:c r="I99" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J99" s="11" t="str">
         <x:v>Le colis est arrivé correctement, même si l'expérience n'avait rien d'exceptionnel.</x:v>
       </x:c>
     </x:row>
@@ -2010,6 +3519,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E100" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F100" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G100" s="16" t="n">
+        <x:v>5.16</x:v>
+      </x:c>
+      <x:c r="H100" s="18" t="n">
+        <x:v>8.4</x:v>
+      </x:c>
+      <x:c r="I100" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J100" s="11" t="str">
         <x:v>Excellente expérience, tout s'est très bien passé.</x:v>
       </x:c>
     </x:row>
@@ -2027,6 +3551,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E101" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F101" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G101" s="16" t="n">
+        <x:v>2.58</x:v>
+      </x:c>
+      <x:c r="H101" s="18" t="n">
+        <x:v>6.8</x:v>
+      </x:c>
+      <x:c r="I101" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J101" s="11" t="str">
         <x:v>Le service était bon et le colis est arrivé sans dommage.</x:v>
       </x:c>
     </x:row>
@@ -2044,6 +3583,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E102" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F102" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G102" s="16" t="n">
+        <x:v>17.65</x:v>
+      </x:c>
+      <x:c r="H102" s="18" t="n">
+        <x:v>16.14</x:v>
+      </x:c>
+      <x:c r="I102" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J102" s="11" t="str">
         <x:v>Très mauvaise expérience, livraison tardive et colis abîmé à l'arrivée.</x:v>
       </x:c>
     </x:row>
@@ -2061,6 +3615,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E103" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F103" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G103" s="16" t="n">
+        <x:v>5.07</x:v>
+      </x:c>
+      <x:c r="H103" s="18" t="n">
+        <x:v>10.84</x:v>
+      </x:c>
+      <x:c r="I103" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J103" s="11" t="str">
         <x:v>Très bonne expérience, avec une livraison ponctuelle et un colis impeccable.</x:v>
       </x:c>
     </x:row>
@@ -2078,6 +3647,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E104" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F104" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G104" s="16" t="n">
+        <x:v>5.46</x:v>
+      </x:c>
+      <x:c r="H104" s="18" t="n">
+        <x:v>8.59</x:v>
+      </x:c>
+      <x:c r="I104" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J104" s="11" t="str">
         <x:v>Service excellent, colis livré rapidement et sans aucun problème.</x:v>
       </x:c>
     </x:row>
@@ -2095,6 +3679,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E105" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F105" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G105" s="16" t="n">
+        <x:v>0.52</x:v>
+      </x:c>
+      <x:c r="H105" s="18" t="n">
+        <x:v>9.22</x:v>
+      </x:c>
+      <x:c r="I105" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J105" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -2111,7 +3710,22 @@
       <x:c r="D106" s="11" t="str">
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
-      <x:c r="E106" s="11"/>
+      <x:c r="E106" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F106" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G106" s="16" t="n">
+        <x:v>0.48</x:v>
+      </x:c>
+      <x:c r="H106" s="18" t="n">
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="I106" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J106" s="11"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="11" t="str">
@@ -2127,6 +3741,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E107" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F107" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G107" s="16" t="n">
+        <x:v>3.08</x:v>
+      </x:c>
+      <x:c r="H107" s="18" t="n">
+        <x:v>10.81</x:v>
+      </x:c>
+      <x:c r="I107" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J107" s="11" t="str">
         <x:v>Le colis était correct mais la livraison a pris trop de temps.</x:v>
       </x:c>
     </x:row>
@@ -2144,6 +3773,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E108" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F108" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G108" s="16" t="n">
+        <x:v>3.98</x:v>
+      </x:c>
+      <x:c r="H108" s="18" t="n">
+        <x:v>7.67</x:v>
+      </x:c>
+      <x:c r="I108" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J108" s="11" t="str">
         <x:v>Le colis a bien été reçu, avec un léger retard sans conséquence importante.</x:v>
       </x:c>
     </x:row>
@@ -2161,6 +3805,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E109" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F109" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G109" s="16" t="n">
+        <x:v>2.66</x:v>
+      </x:c>
+      <x:c r="H109" s="18" t="n">
+        <x:v>10.55</x:v>
+      </x:c>
+      <x:c r="I109" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J109" s="11" t="str">
         <x:v>Le livreur a été peu professionnel et le colis est arrivé en mauvais état.</x:v>
       </x:c>
     </x:row>
@@ -2178,6 +3837,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E110" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F110" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G110" s="16" t="n">
+        <x:v>0.91</x:v>
+      </x:c>
+      <x:c r="H110" s="18" t="n">
+        <x:v>16.96</x:v>
+      </x:c>
+      <x:c r="I110" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J110" s="11" t="str">
         <x:v>La livraison était correcte, sans problème particulier.</x:v>
       </x:c>
     </x:row>
@@ -2195,6 +3869,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E111" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F111" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G111" s="16" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="H111" s="18" t="n">
+        <x:v>16.53</x:v>
+      </x:c>
+      <x:c r="I111" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J111" s="11" t="str">
         <x:v>Service excellent, colis livré rapidement et sans aucun problème.</x:v>
       </x:c>
     </x:row>
@@ -2212,6 +3901,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E112" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F112" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G112" s="16" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H112" s="18" t="n">
+        <x:v>25.7</x:v>
+      </x:c>
+      <x:c r="I112" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J112" s="11" t="str">
         <x:v>Expérience positive dans l'ensemble, avec un colis reçu proprement et dans les temps.</x:v>
       </x:c>
     </x:row>
@@ -2229,6 +3933,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E113" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F113" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G113" s="16" t="n">
+        <x:v>12.26</x:v>
+      </x:c>
+      <x:c r="H113" s="18" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="I113" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J113" s="11" t="str">
         <x:v>Le service a été mauvais du début à la fin, avec beaucoup de retard et un colis abîmé.</x:v>
       </x:c>
     </x:row>
@@ -2246,6 +3965,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E114" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F114" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G114" s="16" t="n">
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="H114" s="18" t="n">
+        <x:v>19.81</x:v>
+      </x:c>
+      <x:c r="I114" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J114" s="11" t="str">
         <x:v>Le colis est arrivé plus tôt que prévu, parfaitement emballé et en excellent état.</x:v>
       </x:c>
     </x:row>
@@ -2263,6 +3997,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E115" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F115" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G115" s="16" t="n">
+        <x:v>0.58</x:v>
+      </x:c>
+      <x:c r="H115" s="18" t="n">
+        <x:v>5.56</x:v>
+      </x:c>
+      <x:c r="I115" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J115" s="11" t="str">
         <x:v>Livraison un peu tardive mais très bonne prise en charge du livreur.</x:v>
       </x:c>
     </x:row>
@@ -2280,6 +4029,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E116" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F116" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G116" s="16" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="H116" s="18" t="n">
+        <x:v>6.01</x:v>
+      </x:c>
+      <x:c r="I116" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J116" s="11" t="str">
         <x:v>Expérience positive dans l'ensemble, avec un colis reçu proprement et dans les temps.</x:v>
       </x:c>
     </x:row>
@@ -2297,6 +4061,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E117" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F117" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G117" s="16" t="n">
+        <x:v>1.06</x:v>
+      </x:c>
+      <x:c r="H117" s="18" t="n">
+        <x:v>5.86</x:v>
+      </x:c>
+      <x:c r="I117" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J117" s="11" t="str">
         <x:v>Service globalement moyen, ni particulièrement bon ni mauvais.</x:v>
       </x:c>
     </x:row>
@@ -2314,6 +4093,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E118" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F118" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G118" s="16" t="n">
+        <x:v>1.06</x:v>
+      </x:c>
+      <x:c r="H118" s="18" t="n">
+        <x:v>5.86</x:v>
+      </x:c>
+      <x:c r="I118" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J118" s="11" t="str">
         <x:v>Service globalement moyen, ni particulièrement bon ni mauvais.</x:v>
       </x:c>
     </x:row>
@@ -2331,6 +4125,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E119" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F119" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G119" s="16" t="n">
+        <x:v>3.59</x:v>
+      </x:c>
+      <x:c r="H119" s="18" t="n">
+        <x:v>11.13</x:v>
+      </x:c>
+      <x:c r="I119" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J119" s="11" t="str">
         <x:v>Expérience positive dans l'ensemble, avec un colis reçu proprement et dans les temps.</x:v>
       </x:c>
     </x:row>
@@ -2348,6 +4157,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E120" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F120" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G120" s="16" t="n">
+        <x:v>5.3</x:v>
+      </x:c>
+      <x:c r="H120" s="18" t="n">
+        <x:v>17.19</x:v>
+      </x:c>
+      <x:c r="I120" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J120" s="11" t="str">
         <x:v>Le colis est arrivé plus tôt que prévu, parfaitement emballé et en excellent état.</x:v>
       </x:c>
     </x:row>
@@ -2365,6 +4189,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E121" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F121" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G121" s="16" t="n">
+        <x:v>4.97</x:v>
+      </x:c>
+      <x:c r="H121" s="18" t="n">
+        <x:v>8.28</x:v>
+      </x:c>
+      <x:c r="I121" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J121" s="11" t="str">
         <x:v>Excellente expérience, tout s'est très bien passé.</x:v>
       </x:c>
     </x:row>
@@ -2382,6 +4221,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E122" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F122" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G122" s="16" t="n">
+        <x:v>6.93</x:v>
+      </x:c>
+      <x:c r="H122" s="18" t="n">
+        <x:v>9.5</x:v>
+      </x:c>
+      <x:c r="I122" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J122" s="11" t="str">
         <x:v>Le colis était en parfait état, mais le service client a mis du temps à répondre.</x:v>
       </x:c>
     </x:row>
@@ -2399,6 +4253,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E123" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F123" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G123" s="16" t="n">
+        <x:v>5.46</x:v>
+      </x:c>
+      <x:c r="H123" s="18" t="n">
+        <x:v>8.59</x:v>
+      </x:c>
+      <x:c r="I123" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J123" s="11" t="str">
         <x:v>Livraison satisfaisante, colis en bon état et livreur courtois.</x:v>
       </x:c>
     </x:row>
@@ -2416,6 +4285,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E124" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F124" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G124" s="16" t="n">
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="H124" s="18" t="n">
+        <x:v>5.39</x:v>
+      </x:c>
+      <x:c r="I124" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J124" s="11" t="str">
         <x:v>Expérience correcte dans l'ensemble, mais le service client pourrait être plus réactif.</x:v>
       </x:c>
     </x:row>
@@ -2433,6 +4317,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E125" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F125" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G125" s="16" t="n">
+        <x:v>5.17</x:v>
+      </x:c>
+      <x:c r="H125" s="18" t="n">
+        <x:v>12.11</x:v>
+      </x:c>
+      <x:c r="I125" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J125" s="11" t="str">
         <x:v>Le service était bon et le colis est arrivé sans dommage.</x:v>
       </x:c>
     </x:row>
@@ -2449,7 +4348,22 @@
       <x:c r="D126" s="11" t="str">
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
-      <x:c r="E126" s="11"/>
+      <x:c r="E126" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F126" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G126" s="16" t="n">
+        <x:v>6.16</x:v>
+      </x:c>
+      <x:c r="H126" s="18" t="n">
+        <x:v>20.22</x:v>
+      </x:c>
+      <x:c r="I126" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J126" s="11"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="11" t="str">
@@ -2465,6 +4379,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E127" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F127" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G127" s="16" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="H127" s="18" t="n">
+        <x:v>9.58</x:v>
+      </x:c>
+      <x:c r="I127" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J127" s="11" t="str">
         <x:v>Le colis est arrivé intact mais le suivi et le service client n'étaient pas satisfaisants.</x:v>
       </x:c>
     </x:row>
@@ -2482,6 +4411,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E128" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F128" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G128" s="16" t="n">
+        <x:v>12.51</x:v>
+      </x:c>
+      <x:c r="H128" s="18" t="n">
+        <x:v>16.66</x:v>
+      </x:c>
+      <x:c r="I128" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J128" s="11" t="str">
         <x:v>Expérience très insatisfaisante, livraison tardive et mauvaise prise en charge du service client.</x:v>
       </x:c>
     </x:row>
@@ -2499,6 +4443,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E129" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F129" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G129" s="16" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="H129" s="18" t="n">
+        <x:v>14.37</x:v>
+      </x:c>
+      <x:c r="I129" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J129" s="11" t="str">
         <x:v>Je suis plutôt insatisfait, surtout à cause du délai de livraison.</x:v>
       </x:c>
     </x:row>
@@ -2516,6 +4475,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E130" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F130" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G130" s="16" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H130" s="18" t="n">
+        <x:v>5.51</x:v>
+      </x:c>
+      <x:c r="I130" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J130" s="11" t="str">
         <x:v>La livraison s'est mal passée, même si le colis était en bon état.</x:v>
       </x:c>
     </x:row>
@@ -2533,6 +4507,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E131" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F131" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G131" s="16" t="n">
+        <x:v>2.25</x:v>
+      </x:c>
+      <x:c r="H131" s="18" t="n">
+        <x:v>6.6</x:v>
+      </x:c>
+      <x:c r="I131" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J131" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -2550,6 +4539,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E132" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F132" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G132" s="16" t="n">
+        <x:v>4.25</x:v>
+      </x:c>
+      <x:c r="H132" s="18" t="n">
+        <x:v>7.83</x:v>
+      </x:c>
+      <x:c r="I132" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J132" s="11" t="str">
         <x:v>Le livreur était correct, mais le retard de livraison était important.</x:v>
       </x:c>
     </x:row>
@@ -2567,6 +4571,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E133" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F133" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G133" s="16" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="H133" s="18" t="n">
+        <x:v>14.09</x:v>
+      </x:c>
+      <x:c r="I133" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J133" s="11" t="str">
         <x:v>Le colis est arrivé plus tôt que prévu, parfaitement emballé et en excellent état.</x:v>
       </x:c>
     </x:row>
@@ -2584,6 +4603,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E134" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F134" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G134" s="16" t="n">
+        <x:v>4.64</x:v>
+      </x:c>
+      <x:c r="H134" s="18" t="n">
+        <x:v>10.58</x:v>
+      </x:c>
+      <x:c r="I134" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J134" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -2601,6 +4635,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E135" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F135" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G135" s="16" t="n">
+        <x:v>9.21</x:v>
+      </x:c>
+      <x:c r="H135" s="18" t="n">
+        <x:v>17.11</x:v>
+      </x:c>
+      <x:c r="I135" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J135" s="11" t="str">
         <x:v>Très satisfait : livraison rapide, livreur courtois et service client efficace.</x:v>
       </x:c>
     </x:row>
@@ -2618,6 +4667,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E136" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F136" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G136" s="16" t="n">
+        <x:v>0.54</x:v>
+      </x:c>
+      <x:c r="H136" s="18" t="n">
+        <x:v>5.53</x:v>
+      </x:c>
+      <x:c r="I136" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J136" s="11" t="str">
         <x:v>Le colis est arrivé intact mais le suivi et le service client n'étaient pas satisfaisants.</x:v>
       </x:c>
     </x:row>
@@ -2635,6 +4699,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E137" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F137" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G137" s="16" t="n">
+        <x:v>0.78</x:v>
+      </x:c>
+      <x:c r="H137" s="18" t="n">
+        <x:v>9.38</x:v>
+      </x:c>
+      <x:c r="I137" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J137" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -2652,6 +4731,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E138" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F138" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G138" s="16" t="n">
+        <x:v>2.19</x:v>
+      </x:c>
+      <x:c r="H138" s="18" t="n">
+        <x:v>17.76</x:v>
+      </x:c>
+      <x:c r="I138" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J138" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -2669,6 +4763,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E139" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F139" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G139" s="16" t="n">
+        <x:v>1.63</x:v>
+      </x:c>
+      <x:c r="H139" s="18" t="n">
+        <x:v>9.91</x:v>
+      </x:c>
+      <x:c r="I139" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J139" s="11" t="str">
         <x:v>Service excellent, colis livré rapidement et sans aucun problème.</x:v>
       </x:c>
     </x:row>
@@ -2686,6 +4795,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E140" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F140" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G140" s="16" t="n">
+        <x:v>6.35</x:v>
+      </x:c>
+      <x:c r="H140" s="18" t="n">
+        <x:v>11.64</x:v>
+      </x:c>
+      <x:c r="I140" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J140" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -2703,6 +4827,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E141" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F141" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G141" s="16" t="n">
+        <x:v>1.31</x:v>
+      </x:c>
+      <x:c r="H141" s="18" t="n">
+        <x:v>14.71</x:v>
+      </x:c>
+      <x:c r="I141" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J141" s="11" t="str">
         <x:v>Très satisfait : livraison rapide, livreur courtois et service client efficace.</x:v>
       </x:c>
     </x:row>
@@ -2720,6 +4859,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E142" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F142" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G142" s="16" t="n">
+        <x:v>2.54</x:v>
+      </x:c>
+      <x:c r="H142" s="18" t="n">
+        <x:v>6.77</x:v>
+      </x:c>
+      <x:c r="I142" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J142" s="11" t="str">
         <x:v>Bonne prise en charge, livraison correcte et livreur professionnel.</x:v>
       </x:c>
     </x:row>
@@ -2737,6 +4891,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E143" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F143" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G143" s="16" t="n">
+        <x:v>3.86</x:v>
+      </x:c>
+      <x:c r="H143" s="18" t="n">
+        <x:v>7.59</x:v>
+      </x:c>
+      <x:c r="I143" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J143" s="11" t="str">
         <x:v>La livraison s'est mal passée, même si le colis était en bon état.</x:v>
       </x:c>
     </x:row>
@@ -2754,6 +4923,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E144" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F144" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G144" s="16" t="n">
+        <x:v>8.99</x:v>
+      </x:c>
+      <x:c r="H144" s="18" t="n">
+        <x:v>19.47</x:v>
+      </x:c>
+      <x:c r="I144" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J144" s="11" t="str">
         <x:v>Expérience correcte dans l'ensemble, mais le service client pourrait être plus réactif.</x:v>
       </x:c>
     </x:row>
@@ -2771,6 +4955,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E145" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F145" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G145" s="16" t="n">
+        <x:v>2.58</x:v>
+      </x:c>
+      <x:c r="H145" s="18" t="n">
+        <x:v>10.5</x:v>
+      </x:c>
+      <x:c r="I145" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J145" s="11" t="str">
         <x:v>La livraison a été lente et les réponses du service client peu utiles.</x:v>
       </x:c>
     </x:row>
@@ -2788,6 +4987,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E146" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F146" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G146" s="16" t="n">
+        <x:v>4.88</x:v>
+      </x:c>
+      <x:c r="H146" s="18" t="n">
+        <x:v>8.23</x:v>
+      </x:c>
+      <x:c r="I146" s="11" t="str">
+        <x:v>Retourné</x:v>
+      </x:c>
+      <x:c r="J146" s="11" t="str">
         <x:v>Le livreur a été peu professionnel et le colis est arrivé en mauvais état.</x:v>
       </x:c>
     </x:row>
@@ -2805,6 +5019,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E147" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F147" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G147" s="16" t="n">
+        <x:v>4.64</x:v>
+      </x:c>
+      <x:c r="H147" s="18" t="n">
+        <x:v>14.28</x:v>
+      </x:c>
+      <x:c r="I147" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J147" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -2822,6 +5051,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E148" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F148" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G148" s="16" t="n">
+        <x:v>3.81</x:v>
+      </x:c>
+      <x:c r="H148" s="18" t="n">
+        <x:v>18.76</x:v>
+      </x:c>
+      <x:c r="I148" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J148" s="11" t="str">
         <x:v>Je suis pleinement satisfait, le service a été rapide et professionnel.</x:v>
       </x:c>
     </x:row>
@@ -2839,6 +5083,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E149" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F149" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G149" s="16" t="n">
+        <x:v>5.17</x:v>
+      </x:c>
+      <x:c r="H149" s="18" t="n">
+        <x:v>12.11</x:v>
+      </x:c>
+      <x:c r="I149" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J149" s="11" t="str">
         <x:v>Je suis pleinement satisfait, le service a été rapide et professionnel.</x:v>
       </x:c>
     </x:row>
@@ -2856,6 +5115,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E150" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F150" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G150" s="16" t="n">
+        <x:v>3.95</x:v>
+      </x:c>
+      <x:c r="H150" s="18" t="n">
+        <x:v>7.65</x:v>
+      </x:c>
+      <x:c r="I150" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J150" s="11" t="str">
         <x:v>Livraison très rapide, colis en parfait état et livreur très professionnel.</x:v>
       </x:c>
     </x:row>
@@ -2873,6 +5147,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E151" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F151" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G151" s="16" t="n">
+        <x:v>4.42</x:v>
+      </x:c>
+      <x:c r="H151" s="18" t="n">
+        <x:v>19.14</x:v>
+      </x:c>
+      <x:c r="I151" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J151" s="11" t="str">
         <x:v>Bonne expérience dans l'ensemble, malgré un léger retard.</x:v>
       </x:c>
     </x:row>
@@ -2890,6 +5179,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E152" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F152" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G152" s="16" t="n">
+        <x:v>1.22</x:v>
+      </x:c>
+      <x:c r="H152" s="18" t="n">
+        <x:v>14.66</x:v>
+      </x:c>
+      <x:c r="I152" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J152" s="11" t="str">
         <x:v>Le colis est arrivé plusieurs jours en retard et le support n'a pas résolu mon problème.</x:v>
       </x:c>
     </x:row>
@@ -2907,6 +5211,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E153" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F153" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G153" s="16" t="n">
+        <x:v>1.28</x:v>
+      </x:c>
+      <x:c r="H153" s="18" t="n">
+        <x:v>8.49</x:v>
+      </x:c>
+      <x:c r="I153" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J153" s="11" t="str">
         <x:v>Excellente expérience, tout s'est très bien passé.</x:v>
       </x:c>
     </x:row>
@@ -2924,6 +5243,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E154" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F154" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G154" s="16" t="n">
+        <x:v>4.31</x:v>
+      </x:c>
+      <x:c r="H154" s="18" t="n">
+        <x:v>11.57</x:v>
+      </x:c>
+      <x:c r="I154" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J154" s="11" t="str">
         <x:v>Service globalement moyen, ni particulièrement bon ni mauvais.</x:v>
       </x:c>
     </x:row>
@@ -2941,6 +5275,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E155" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F155" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G155" s="16" t="n">
+        <x:v>4.75</x:v>
+      </x:c>
+      <x:c r="H155" s="18" t="n">
+        <x:v>14.35</x:v>
+      </x:c>
+      <x:c r="I155" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J155" s="11" t="str">
         <x:v>Le colis est arrivé intact mais le suivi et le service client n'étaient pas satisfaisants.</x:v>
       </x:c>
     </x:row>
@@ -2958,6 +5307,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E156" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F156" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G156" s="16" t="n">
+        <x:v>0.71</x:v>
+      </x:c>
+      <x:c r="H156" s="18" t="n">
+        <x:v>5.64</x:v>
+      </x:c>
+      <x:c r="I156" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J156" s="11" t="str">
         <x:v>Le colis est arrivé intact mais le suivi et le service client n'étaient pas satisfaisants.</x:v>
       </x:c>
     </x:row>
@@ -2975,6 +5339,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E157" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F157" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G157" s="16" t="n">
+        <x:v>5.18</x:v>
+      </x:c>
+      <x:c r="H157" s="18" t="n">
+        <x:v>8.41</x:v>
+      </x:c>
+      <x:c r="I157" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J157" s="11" t="str">
         <x:v>Le colis est arrivé avec du retard et le service client était difficile à joindre.</x:v>
       </x:c>
     </x:row>
@@ -2992,6 +5371,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E158" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F158" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G158" s="16" t="n">
+        <x:v>5.33</x:v>
+      </x:c>
+      <x:c r="H158" s="18" t="n">
+        <x:v>8.5</x:v>
+      </x:c>
+      <x:c r="I158" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J158" s="11" t="str">
         <x:v>Expérience positive dans l'ensemble, avec un colis reçu proprement et dans les temps.</x:v>
       </x:c>
     </x:row>
@@ -3009,6 +5403,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E159" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F159" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G159" s="16" t="n">
+        <x:v>16.1</x:v>
+      </x:c>
+      <x:c r="H159" s="18" t="n">
+        <x:v>21.38</x:v>
+      </x:c>
+      <x:c r="I159" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J159" s="11" t="str">
         <x:v>Expérience correcte dans l'ensemble, mais le service client pourrait être plus réactif.</x:v>
       </x:c>
     </x:row>
@@ -3026,6 +5435,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E160" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F160" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G160" s="16" t="n">
+        <x:v>1.12</x:v>
+      </x:c>
+      <x:c r="H160" s="18" t="n">
+        <x:v>8.39</x:v>
+      </x:c>
+      <x:c r="I160" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J160" s="11" t="str">
         <x:v>Le colis est arrivé plus tôt que prévu, parfaitement emballé et en excellent état.</x:v>
       </x:c>
     </x:row>
@@ -3043,6 +5467,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E161" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F161" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G161" s="16" t="n">
+        <x:v>1.79</x:v>
+      </x:c>
+      <x:c r="H161" s="18" t="n">
+        <x:v>10.01</x:v>
+      </x:c>
+      <x:c r="I161" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J161" s="11" t="str">
         <x:v>Livraison très rapide, colis en parfait état et livreur très professionnel.</x:v>
       </x:c>
     </x:row>
@@ -3060,6 +5499,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E162" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F162" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G162" s="16" t="n">
+        <x:v>0.89</x:v>
+      </x:c>
+      <x:c r="H162" s="18" t="n">
+        <x:v>8.25</x:v>
+      </x:c>
+      <x:c r="I162" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J162" s="11" t="str">
         <x:v>Très satisfait : livraison rapide, livreur courtois et service client efficace.</x:v>
       </x:c>
     </x:row>
@@ -3077,6 +5531,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E163" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F163" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G163" s="16" t="n">
+        <x:v>1.26</x:v>
+      </x:c>
+      <x:c r="H163" s="18" t="n">
+        <x:v>8.48</x:v>
+      </x:c>
+      <x:c r="I163" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J163" s="11" t="str">
         <x:v>Le colis est arrivé correctement, même si l'expérience n'avait rien d'exceptionnel.</x:v>
       </x:c>
     </x:row>
@@ -3094,6 +5563,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E164" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F164" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G164" s="16" t="n">
+        <x:v>0.38</x:v>
+      </x:c>
+      <x:c r="H164" s="18" t="n">
+        <x:v>16.64</x:v>
+      </x:c>
+      <x:c r="I164" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J164" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -3111,6 +5595,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E165" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F165" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G165" s="16" t="n">
+        <x:v>0.77</x:v>
+      </x:c>
+      <x:c r="H165" s="18" t="n">
+        <x:v>5.68</x:v>
+      </x:c>
+      <x:c r="I165" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J165" s="11" t="str">
         <x:v>Le colis est arrivé à temps et le livreur était professionnel.</x:v>
       </x:c>
     </x:row>
@@ -3128,6 +5627,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E166" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F166" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G166" s="16" t="n">
+        <x:v>5.25</x:v>
+      </x:c>
+      <x:c r="H166" s="18" t="n">
+        <x:v>8.46</x:v>
+      </x:c>
+      <x:c r="I166" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J166" s="11" t="str">
         <x:v>Livraison satisfaisante, colis en bon état et livreur courtois.</x:v>
       </x:c>
     </x:row>
@@ -3145,6 +5659,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E167" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F167" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G167" s="16" t="n">
+        <x:v>1.27</x:v>
+      </x:c>
+      <x:c r="H167" s="18" t="n">
+        <x:v>5.99</x:v>
+      </x:c>
+      <x:c r="I167" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J167" s="11" t="str">
         <x:v>Service excellent, colis livré rapidement et sans aucun problème.</x:v>
       </x:c>
     </x:row>
@@ -3162,6 +5691,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E168" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F168" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G168" s="16" t="n">
+        <x:v>0.51</x:v>
+      </x:c>
+      <x:c r="H168" s="18" t="n">
+        <x:v>11.72</x:v>
+      </x:c>
+      <x:c r="I168" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J168" s="11" t="str">
         <x:v>Le service était bon et le colis est arrivé sans dommage.</x:v>
       </x:c>
     </x:row>
@@ -3179,6 +5723,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E169" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F169" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G169" s="16" t="n">
+        <x:v>2.78</x:v>
+      </x:c>
+      <x:c r="H169" s="18" t="n">
+        <x:v>6.92</x:v>
+      </x:c>
+      <x:c r="I169" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J169" s="11" t="str">
         <x:v>Le colis est arrivé plus tôt que prévu, parfaitement emballé et en excellent état.</x:v>
       </x:c>
     </x:row>
@@ -3196,6 +5755,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E170" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F170" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G170" s="16" t="n">
+        <x:v>5.61</x:v>
+      </x:c>
+      <x:c r="H170" s="18" t="n">
+        <x:v>8.68</x:v>
+      </x:c>
+      <x:c r="I170" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J170" s="11" t="str">
         <x:v>Je suis pleinement satisfait, le service a été rapide et professionnel.</x:v>
       </x:c>
     </x:row>
@@ -3213,6 +5787,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E171" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F171" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G171" s="16" t="n">
+        <x:v>4.49</x:v>
+      </x:c>
+      <x:c r="H171" s="18" t="n">
+        <x:v>19.18</x:v>
+      </x:c>
+      <x:c r="I171" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J171" s="11" t="str">
         <x:v>Le livreur était professionnel mais le colis est arrivé en retard.</x:v>
       </x:c>
     </x:row>
@@ -3230,6 +5819,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E172" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F172" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G172" s="16" t="n">
+        <x:v>0.89</x:v>
+      </x:c>
+      <x:c r="H172" s="18" t="n">
+        <x:v>9.45</x:v>
+      </x:c>
+      <x:c r="I172" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J172" s="11" t="str">
         <x:v>Je suis pleinement satisfait, le service a été rapide et professionnel.</x:v>
       </x:c>
     </x:row>
@@ -3247,6 +5851,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E173" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F173" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G173" s="16" t="n">
+        <x:v>1.03</x:v>
+      </x:c>
+      <x:c r="H173" s="18" t="n">
+        <x:v>5.84</x:v>
+      </x:c>
+      <x:c r="I173" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J173" s="11" t="str">
         <x:v>La livraison s'est passée normalement et le colis était en bon état.</x:v>
       </x:c>
     </x:row>
@@ -3264,6 +5883,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E174" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F174" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G174" s="16" t="n">
+        <x:v>12.13</x:v>
+      </x:c>
+      <x:c r="H174" s="18" t="n">
+        <x:v>16.42</x:v>
+      </x:c>
+      <x:c r="I174" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J174" s="11" t="str">
         <x:v>Livraison satisfaisante, colis en bon état et livreur courtois.</x:v>
       </x:c>
     </x:row>
@@ -3281,6 +5915,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E175" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F175" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G175" s="16" t="n">
+        <x:v>0.31</x:v>
+      </x:c>
+      <x:c r="H175" s="18" t="n">
+        <x:v>7.89</x:v>
+      </x:c>
+      <x:c r="I175" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J175" s="11" t="str">
         <x:v>Le service était bon et le colis est arrivé sans dommage.</x:v>
       </x:c>
     </x:row>
@@ -3298,6 +5947,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E176" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F176" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G176" s="16" t="n">
+        <x:v>1.41</x:v>
+      </x:c>
+      <x:c r="H176" s="18" t="n">
+        <x:v>6.07</x:v>
+      </x:c>
+      <x:c r="I176" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J176" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -3315,6 +5979,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E177" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F177" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G177" s="16" t="n">
+        <x:v>10.88</x:v>
+      </x:c>
+      <x:c r="H177" s="18" t="n">
+        <x:v>11.95</x:v>
+      </x:c>
+      <x:c r="I177" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J177" s="11" t="str">
         <x:v>Le colis a bien été reçu, avec un léger retard sans conséquence importante.</x:v>
       </x:c>
     </x:row>
@@ -3332,6 +6011,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E178" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F178" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G178" s="16" t="n">
+        <x:v>3.66</x:v>
+      </x:c>
+      <x:c r="H178" s="18" t="n">
+        <x:v>13.67</x:v>
+      </x:c>
+      <x:c r="I178" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J178" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -3349,6 +6043,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E179" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F179" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G179" s="16" t="n">
+        <x:v>1.38</x:v>
+      </x:c>
+      <x:c r="H179" s="18" t="n">
+        <x:v>8.56</x:v>
+      </x:c>
+      <x:c r="I179" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J179" s="11" t="str">
         <x:v>Tout était parfait, de la livraison à l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -3366,6 +6075,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E180" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F180" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G180" s="16" t="n">
+        <x:v>3.59</x:v>
+      </x:c>
+      <x:c r="H180" s="18" t="n">
+        <x:v>13.63</x:v>
+      </x:c>
+      <x:c r="I180" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J180" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -3383,6 +6107,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E181" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F181" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G181" s="16" t="n">
+        <x:v>16.37</x:v>
+      </x:c>
+      <x:c r="H181" s="18" t="n">
+        <x:v>26.55</x:v>
+      </x:c>
+      <x:c r="I181" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J181" s="11" t="str">
         <x:v>Le colis est arrivé avec du retard et le service client était difficile à joindre.</x:v>
       </x:c>
     </x:row>
@@ -3400,6 +6139,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E182" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F182" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G182" s="16" t="n">
+        <x:v>3.25</x:v>
+      </x:c>
+      <x:c r="H182" s="18" t="n">
+        <x:v>7.21</x:v>
+      </x:c>
+      <x:c r="I182" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J182" s="11" t="str">
         <x:v>La livraison s'est passée normalement et le colis était en bon état.</x:v>
       </x:c>
     </x:row>
@@ -3417,6 +6171,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E183" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F183" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G183" s="16" t="n">
+        <x:v>15.94</x:v>
+      </x:c>
+      <x:c r="H183" s="18" t="n">
+        <x:v>15.08</x:v>
+      </x:c>
+      <x:c r="I183" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J183" s="11" t="str">
         <x:v>Bonne prise en charge, livraison correcte et livreur professionnel.</x:v>
       </x:c>
     </x:row>
@@ -3434,6 +6203,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E184" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F184" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G184" s="16" t="n">
+        <x:v>6.55</x:v>
+      </x:c>
+      <x:c r="H184" s="18" t="n">
+        <x:v>20.46</x:v>
+      </x:c>
+      <x:c r="I184" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J184" s="11" t="str">
         <x:v>Livraison satisfaisante, colis en bon état et livreur courtois.</x:v>
       </x:c>
     </x:row>
@@ -3451,6 +6235,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E185" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F185" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G185" s="16" t="n">
+        <x:v>4.71</x:v>
+      </x:c>
+      <x:c r="H185" s="18" t="n">
+        <x:v>8.12</x:v>
+      </x:c>
+      <x:c r="I185" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J185" s="11" t="str">
         <x:v>Livraison très rapide, colis en parfait état et livreur très professionnel.</x:v>
       </x:c>
     </x:row>
@@ -3468,6 +6267,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E186" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F186" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G186" s="16" t="n">
+        <x:v>1.19</x:v>
+      </x:c>
+      <x:c r="H186" s="18" t="n">
+        <x:v>14.64</x:v>
+      </x:c>
+      <x:c r="I186" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J186" s="11" t="str">
         <x:v>Expérience positive dans l'ensemble, avec un colis reçu proprement et dans les temps.</x:v>
       </x:c>
     </x:row>
@@ -3485,6 +6299,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E187" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F187" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G187" s="16" t="n">
+        <x:v>5.65</x:v>
+      </x:c>
+      <x:c r="H187" s="18" t="n">
+        <x:v>8.7</x:v>
+      </x:c>
+      <x:c r="I187" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J187" s="11" t="str">
         <x:v>Livraison satisfaisante, colis en bon état et livreur courtois.</x:v>
       </x:c>
     </x:row>
@@ -3502,6 +6331,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E188" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F188" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G188" s="16" t="n">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="H188" s="18" t="n">
+        <x:v>14.49</x:v>
+      </x:c>
+      <x:c r="I188" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J188" s="11" t="str">
         <x:v>La livraison était correcte, sans problème particulier.</x:v>
       </x:c>
     </x:row>
@@ -3519,6 +6363,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E189" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F189" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G189" s="16" t="n">
+        <x:v>2.24</x:v>
+      </x:c>
+      <x:c r="H189" s="18" t="n">
+        <x:v>6.59</x:v>
+      </x:c>
+      <x:c r="I189" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J189" s="11" t="str">
         <x:v>Je suis pleinement satisfait, le service a été rapide et professionnel.</x:v>
       </x:c>
     </x:row>
@@ -3536,6 +6395,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E190" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F190" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G190" s="16" t="n">
+        <x:v>4.14</x:v>
+      </x:c>
+      <x:c r="H190" s="18" t="n">
+        <x:v>18.97</x:v>
+      </x:c>
+      <x:c r="I190" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J190" s="11" t="str">
         <x:v>Expérience correcte dans l'ensemble, mais le service client pourrait être plus réactif.</x:v>
       </x:c>
     </x:row>
@@ -3553,6 +6427,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E191" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F191" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G191" s="16" t="n">
+        <x:v>7.21</x:v>
+      </x:c>
+      <x:c r="H191" s="18" t="n">
+        <x:v>20.87</x:v>
+      </x:c>
+      <x:c r="I191" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J191" s="11" t="str">
         <x:v>Le colis est arrivé à temps et le livreur était professionnel.</x:v>
       </x:c>
     </x:row>
@@ -3570,6 +6459,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E192" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F192" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G192" s="16" t="n">
+        <x:v>11.43</x:v>
+      </x:c>
+      <x:c r="H192" s="18" t="n">
+        <x:v>12.29</x:v>
+      </x:c>
+      <x:c r="I192" s="11" t="str">
+        <x:v>En transit</x:v>
+      </x:c>
+      <x:c r="J192" s="11" t="str">
         <x:v>Le colis est arrivé intact mais le suivi et le service client n'étaient pas satisfaisants.</x:v>
       </x:c>
     </x:row>
@@ -3587,6 +6491,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E193" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F193" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G193" s="16" t="n">
+        <x:v>5.14</x:v>
+      </x:c>
+      <x:c r="H193" s="18" t="n">
+        <x:v>10.89</x:v>
+      </x:c>
+      <x:c r="I193" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J193" s="11" t="str">
         <x:v>Le colis est arrivé dans un état correct, mais le délai était un peu long.</x:v>
       </x:c>
     </x:row>
@@ -3604,6 +6523,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E194" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F194" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G194" s="16" t="n">
+        <x:v>5.79</x:v>
+      </x:c>
+      <x:c r="H194" s="18" t="n">
+        <x:v>8.79</x:v>
+      </x:c>
+      <x:c r="I194" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J194" s="11" t="str">
         <x:v>Tout était parfait, de la livraison à l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -3620,7 +6554,22 @@
       <x:c r="D195" s="11" t="str">
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
-      <x:c r="E195" s="11"/>
+      <x:c r="E195" s="11" t="str">
+        <x:v>Grand</x:v>
+      </x:c>
+      <x:c r="F195" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G195" s="16" t="n">
+        <x:v>8.55</x:v>
+      </x:c>
+      <x:c r="H195" s="18" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="I195" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J195" s="11"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="11" t="str">
@@ -3636,6 +6585,21 @@
         <x:v>COLIS_PREMIUM</x:v>
       </x:c>
       <x:c r="E196" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F196" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G196" s="16" t="n">
+        <x:v>0.62</x:v>
+      </x:c>
+      <x:c r="H196" s="18" t="n">
+        <x:v>16.78</x:v>
+      </x:c>
+      <x:c r="I196" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J196" s="11" t="str">
         <x:v>La livraison a été lente et les réponses du service client peu utiles.</x:v>
       </x:c>
     </x:row>
@@ -3653,6 +6617,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E197" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F197" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G197" s="16" t="n">
+        <x:v>1.46</x:v>
+      </x:c>
+      <x:c r="H197" s="18" t="n">
+        <x:v>8.61</x:v>
+      </x:c>
+      <x:c r="I197" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J197" s="11" t="str">
         <x:v>Je suis très déçu : le colis a été livré tard et en mauvais état.</x:v>
       </x:c>
     </x:row>
@@ -3670,6 +6649,21 @@
         <x:v>COLIS_EXPRESS</x:v>
       </x:c>
       <x:c r="E198" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F198" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G198" s="16" t="n">
+        <x:v>5.6</x:v>
+      </x:c>
+      <x:c r="H198" s="18" t="n">
+        <x:v>12.37</x:v>
+      </x:c>
+      <x:c r="I198" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J198" s="11" t="str">
         <x:v>Expérience très insatisfaisante, livraison tardive et mauvaise prise en charge du service client.</x:v>
       </x:c>
     </x:row>
@@ -3687,6 +6681,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E199" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F199" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G199" s="16" t="n">
+        <x:v>4.63</x:v>
+      </x:c>
+      <x:c r="H199" s="18" t="n">
+        <x:v>10.57</x:v>
+      </x:c>
+      <x:c r="I199" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J199" s="11" t="str">
         <x:v>Très bonne expérience, avec une livraison ponctuelle et un colis impeccable.</x:v>
       </x:c>
     </x:row>
@@ -3704,6 +6713,21 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E200" s="11" t="str">
+        <x:v>Moyen</x:v>
+      </x:c>
+      <x:c r="F200" s="11" t="str">
+        <x:v>Non</x:v>
+      </x:c>
+      <x:c r="G200" s="16" t="n">
+        <x:v>2.57</x:v>
+      </x:c>
+      <x:c r="H200" s="18" t="n">
+        <x:v>6.79</x:v>
+      </x:c>
+      <x:c r="I200" s="11" t="str">
+        <x:v>Livré</x:v>
+      </x:c>
+      <x:c r="J200" s="11" t="str">
         <x:v>Tout était parfait, de la livraison à l'état du colis.</x:v>
       </x:c>
     </x:row>
@@ -3721,18 +6745,33 @@
         <x:v>COLIS_STANDARD</x:v>
       </x:c>
       <x:c r="E201" s="11" t="str">
+        <x:v>Petit</x:v>
+      </x:c>
+      <x:c r="F201" s="11" t="str">
+        <x:v>Oui</x:v>
+      </x:c>
+      <x:c r="G201" s="16" t="n">
+        <x:v>1.37</x:v>
+      </x:c>
+      <x:c r="H201" s="18" t="n">
+        <x:v>8.55</x:v>
+      </x:c>
+      <x:c r="I201" s="11" t="str">
+        <x:v>Retardé</x:v>
+      </x:c>
+      <x:c r="J201" s="11" t="str">
         <x:v>Je suis satisfait de la livraison et de l'état du colis.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="E2:E201">
+  <x:conditionalFormatting sqref="J2:J201">
     <x:cfRule type="expression" dxfId="0" priority="1">
-      <x:formula>ISBLANK(E2)</x:formula>
+      <x:formula>ISBLANK(J2)</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb0953618abe47d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ad6b8d0253445a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3741,28 +6780,28 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="78" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="18" t="str">
+      <x:c r="A1" s="22" t="str">
         <x:v>Jeu de données</x:v>
       </x:c>
-      <x:c r="B1" s="18" t="str">
+      <x:c r="B1" s="22" t="str">
         <x:v>FastColis Maroc - Enquêtes fictives de satisfaction</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="16" t="str">
-        <x:v>Nombre d'enquêtes</x:v>
+      <x:c r="A2" s="20" t="str">
+        <x:v>Nombre de lignes</x:v>
       </x:c>
       <x:c r="B2" t="n">
         <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="16" t="str">
+      <x:c r="A3" s="20" t="str">
         <x:v>Période</x:v>
       </x:c>
       <x:c r="B3" t="str">
@@ -3770,7 +6809,7 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="16" t="str">
+      <x:c r="A4" s="20" t="str">
         <x:v>Pays</x:v>
       </x:c>
       <x:c r="B4" t="str">
@@ -3778,59 +6817,99 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="16" t="str">
+      <x:c r="A5" s="20" t="str">
         <x:v>Format de satisfaction</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Un commentaire global en texte libre par colis</x:v>
+        <x:v>Un commentaire_global en texte libre par colis</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="16" t="str">
-        <x:v>Objectif NLP/LLM</x:v>
+      <x:c r="A6" s="20" t="str">
+        <x:v>Note de satisfaction</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Transformer ultérieurement chaque commentaire en une note de satisfaction de 1 à 5</x:v>
+        <x:v>Aucune note n'est créée dans cette source</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="16" t="str">
+      <x:c r="A7" s="20" t="str">
         <x:v>Commentaires manquants</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>10 commentaires manquants, soit 5 % des enquêtes</x:v>
+        <x:v>10 commentaires manquants conservés</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="16" t="str">
-        <x:v>Doublons logiques</x:v>
+      <x:c r="A8" s="20" t="str">
+        <x:v>Nouvelles colonnes</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>6 profils d'enquête dupliqués avec un id_enquete différent</x:v>
+        <x:v>taille_colis, fragile, poids_kg, prix_livraison_eur, statut_colis</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="16" t="str">
-        <x:v>Commentaires contradictoires</x:v>
+      <x:c r="A9" s="20" t="str">
+        <x:v>taille_colis</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>8 commentaires légèrement mixtes pour tester la robustesse du traitement NLP</x:v>
+        <x:v>Petit, Moyen ou Grand</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="16" t="str">
+      <x:c r="A10" s="20" t="str">
+        <x:v>fragile</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Oui ou Non</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="20" t="str">
+        <x:v>poids_kg</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Poids réaliste cohérent avec la taille du colis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="20" t="str">
+        <x:v>prix_livraison_eur</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Prix cohérent avec le produit, le poids et la fragilité</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="20" t="str">
+        <x:v>statut_colis</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Livré, En transit, Retardé ou Retourné</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="20" t="str">
+        <x:v>commentaire_global</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Commentaire d'origine conservé pour une future classification NLP / LLM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="20" t="str">
         <x:v>Données personnelles</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="B15" t="str">
         <x:v>Aucune donnée personnelle réelle</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="16" t="str">
-        <x:v>Important</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>Aucune note de satisfaction n'est stockée dans le dataset</x:v>
+    <x:row r="16">
+      <x:c r="A16" s="20" t="str">
+        <x:v>Objectif</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Tester ingestion, profiling, qualité, nettoyage, standardisation puis classification du texte</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>